<commit_message>
Publish sanitized Excel baseline v2
</commit_message>
<xml_diff>
--- a/Lets Meet DB Dump.xlsx
+++ b/Lets Meet DB Dump.xlsx
@@ -3926,7 +3926,7 @@
     <t>06221 / 98689</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %57%; Mir die Probleme von anderen anhören %21%; Abends seinem Partner Ereignisse des Tages erzählen %53%; Für einen guten Zweck spenden %25%; </t>
+    <t xml:space="preserve">Für jemanden kochen %57%; Mir die Probleme von anderen anhören %21%; Abends seinem Partner Ereignisse des Tages erzählen %53%; Für einen guten Zweck spenden %25%; </t>
   </si>
   <si>
     <t>tsanaklidou.elina@1mal1.te</t>
@@ -4157,7 +4157,7 @@
     <t>09396 / 11522</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %1%; Einfach mit guten Freunden zwanglos plaudern %28%; Entspannungsübungen machen %69%; Ein Nickerchen machen %31%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %1%; Einfach mit guten Freunden zwanglos plaudern %28%; Entspannungsübungen machen %69%; Ein Nickerchen machen %31%; </t>
   </si>
   <si>
     <t>georgios.wijnenriems@iunitimail.ork</t>
@@ -4229,7 +4229,7 @@
     <t>07102 / 41073</t>
   </si>
   <si>
-    <t xml:space="preserve">Motorrad fahren %84%; Seine Haare waschen %42%; Etwas planen oder organisieren %2%; </t>
+    <t xml:space="preserve">Motorrad fahren %84%; Seine Fotos sortieren %42%; Etwas planen oder organisieren %2%; </t>
   </si>
   <si>
     <t>dariusz-robert.seliger@web.kom</t>
@@ -5192,7 +5192,7 @@
     <t>(03328) 21759</t>
   </si>
   <si>
-    <t xml:space="preserve">In ein Lokal gehen %64%; E-Mails schreiben %42%; Musik hören %56%; Eine Dusche nehmen %38%; </t>
+    <t xml:space="preserve">In ein Lokal gehen %64%; E-Mails schreiben %42%; Musik hören %56%; Frische Luft schnappen %38%; </t>
   </si>
   <si>
     <t>stephan.janek@web.kom</t>
@@ -5471,7 +5471,7 @@
     <t>(0168) 25014</t>
   </si>
   <si>
-    <t xml:space="preserve">Zu einem Frisör oder Kosmetiker gehen %10%; Sich politisch oder sozial betätigen %24%; Über meine Interessen diskutieren %96%; Mich schön kleiden %67%; Eine Dusche nehmen %49%; </t>
+    <t xml:space="preserve">Zu einem Frisör oder Kosmetiker gehen %10%; Sich politisch oder sozial betätigen %24%; Über meine Interessen diskutieren %96%; Mich schön kleiden %67%; Frische Luft schnappen %49%; </t>
   </si>
   <si>
     <t>tamer.behling@web.te</t>
@@ -5714,7 +5714,7 @@
     <t>04103 / 40015</t>
   </si>
   <si>
-    <t xml:space="preserve">Kräuter/Pilze sammeln %71%; Ausgiebig baden %94%; Auf mich zukommende Situationen in Gedanken bewältigen %71%; </t>
+    <t xml:space="preserve">Kräuter/Pilze sammeln %71%; Ausgiebig Tee trinken %94%; Auf mich zukommende Situationen in Gedanken bewältigen %71%; </t>
   </si>
   <si>
     <t>thomas.prenger-berninghoff@ge-em-ix.ork</t>
@@ -5765,7 +5765,7 @@
     <t>0208 / 467903</t>
   </si>
   <si>
-    <t xml:space="preserve">Zu Gerichtsverhandlungen gehen %45%; Morgens Früh aufstehen %0%; Eine Dusche nehmen %44%; </t>
+    <t xml:space="preserve">Zu Gerichtsverhandlungen gehen %45%; Morgens Früh aufstehen %0%; Frische Luft schnappen %44%; </t>
   </si>
   <si>
     <t>šešlija.marija@autluuk.te</t>
@@ -5840,7 +5840,7 @@
     <t>02177 / 74848</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich über Philosophie oder Religion unterhalten %41%; Schwierige Probleme klären %31%; Malen, basteln, musizieren, usw. %9%; Eine Dusche nehmen %84%; </t>
+    <t xml:space="preserve">Sich über Philosophie oder Religion unterhalten %41%; Schwierige Probleme klären %31%; Malen, basteln, musizieren, usw. %9%; Frische Luft schnappen %84%; </t>
   </si>
   <si>
     <t>paul.degelmann@web.te</t>
@@ -5900,7 +5900,7 @@
     <t>0521 / 725539</t>
   </si>
   <si>
-    <t xml:space="preserve">Kartenspielen %93%; E-Mails schreiben %25%; Einen Spaziergang machen %43%; Eine Dusche nehmen %15%; </t>
+    <t xml:space="preserve">Kartenspielen %93%; E-Mails schreiben %25%; Einen Spaziergang machen %43%; Frische Luft schnappen %15%; </t>
   </si>
   <si>
     <t>jürgen.müller@web.te</t>
@@ -5975,7 +5975,7 @@
     <t>03301 / 29486</t>
   </si>
   <si>
-    <t xml:space="preserve">Möglichst pünktlich wegkommen %0%; Seine Haare waschen %35%; Etwas lernen und mich fortbilden %23%; </t>
+    <t xml:space="preserve">Möglichst pünktlich wegkommen %0%; Seine Fotos sortieren %35%; Etwas lernen und mich fortbilden %23%; </t>
   </si>
   <si>
     <t>udo.hutschenreiter@d-ohnline.kom</t>
@@ -6338,7 +6338,7 @@
     <t>05445 / 12746</t>
   </si>
   <si>
-    <t xml:space="preserve">Reiten %18%; Meine Arbeit geschickt ausführen %81%; Über die Probleme anderer Leute nachdenken %6%; Eine Dusche nehmen %30%; </t>
+    <t xml:space="preserve">Reiten %18%; Meine Arbeit geschickt ausführen %81%; Über die Probleme anderer Leute nachdenken %6%; Frische Luft schnappen %30%; </t>
   </si>
   <si>
     <t>maria.peters@1mal1.te</t>
@@ -6632,7 +6632,7 @@
     <t>02725 / 92431</t>
   </si>
   <si>
-    <t xml:space="preserve">Erkundungsgänge machen (unbekannte Gegenden) %59%; Kartenspielen %52%; Über meine Interessen diskutieren %19%; Kochen oder backen %37%; Eine Dusche nehmen %82%; </t>
+    <t xml:space="preserve">Erkundungsgänge machen (unbekannte Gegenden) %59%; Kartenspielen %52%; Über meine Interessen diskutieren %19%; Kochen oder backen %37%; Frische Luft schnappen %82%; </t>
   </si>
   <si>
     <t>06.08.1974</t>
@@ -6818,7 +6818,7 @@
     <t>05971 / 6680</t>
   </si>
   <si>
-    <t xml:space="preserve">Ins Grüne fahren %28%; Zärtlich sein, schmusen, küssen %13%; Schwierige Probleme klären %52%; Abends seinem Partner Ereignisse des Tages erzählen %66%; Eine Dusche nehmen %82%; </t>
+    <t xml:space="preserve">Ins Grüne fahren %28%; Einen gemütlichen Filmabend machen %13%; Schwierige Probleme klären %52%; Abends seinem Partner Ereignisse des Tages erzählen %66%; Frische Luft schnappen %82%; </t>
   </si>
   <si>
     <t>huber.elisabeth@iunitimail.te</t>
@@ -7100,7 +7100,7 @@
     <t>(0162) 485828</t>
   </si>
   <si>
-    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %63%; Ausgiebig baden %76%; </t>
+    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %63%; Ausgiebig Tee trinken %76%; </t>
   </si>
   <si>
     <t>erwin.bangel@d-ohnline.te</t>
@@ -7163,7 +7163,7 @@
     <t>0162 280648</t>
   </si>
   <si>
-    <t xml:space="preserve">Gymnastik, Fitnessübungen betreiben %46%; Eine Blume oder Pflanze sehen oder daran riechen %75%; Eine Dusche nehmen %30%; </t>
+    <t xml:space="preserve">Gymnastik, Fitnessübungen betreiben %46%; Eine Blume oder Pflanze sehen oder daran riechen %75%; Frische Luft schnappen %30%; </t>
   </si>
   <si>
     <t>maria-analia.ballmann@autluuk.te</t>
@@ -7415,7 +7415,7 @@
     <t>0541 / 706278</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich beruflich engagieren %52%; Faulenzen %24%; Eine Dusche nehmen %52%; </t>
+    <t xml:space="preserve">Sich beruflich engagieren %52%; Faulenzen %24%; Frische Luft schnappen %52%; </t>
   </si>
   <si>
     <t>hiltrud.pacla@web.te</t>
@@ -7541,7 +7541,7 @@
     <t>05345 / 99473</t>
   </si>
   <si>
-    <t xml:space="preserve">Über Politik oder öffentliche Angelegenheiten reden %79%; Um Hilfe und Ratschläge bitten %66%; Seine Haare waschen %12%; Antiquitäten restaurieren, Möbel aufarbeiten %54%; </t>
+    <t xml:space="preserve">Über Politik oder öffentliche Angelegenheiten reden %79%; Um Hilfe und Ratschläge bitten %66%; Seine Fotos sortieren %12%; Antiquitäten restaurieren, Möbel aufarbeiten %54%; </t>
   </si>
   <si>
     <t>ute.newels@d-ohnline.te</t>
@@ -7754,7 +7754,7 @@
     <t>0361 / 816312</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %60%; Mir selbst etwas kochen %62%; Etwas entwerfen oder zeichnen %30%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %60%; Mir selbst etwas kochen %62%; Etwas entwerfen oder zeichnen %30%; </t>
   </si>
   <si>
     <t>davinio.giuseppe@d-ohnline.te</t>
@@ -7850,7 +7850,7 @@
     <t>(04161) 32085</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich mit Tieren beschäftigen %86%; Zärtlich sein, schmusen, küssen %8%; Post lesen %52%; </t>
+    <t xml:space="preserve">Sich mit Tieren beschäftigen %86%; Einen gemütlichen Filmabend machen %8%; Post lesen %52%; </t>
   </si>
   <si>
     <t>işık.sayar@iunitimail.kom</t>
@@ -8357,7 +8357,7 @@
     <t>0209 / 572079</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit Partner oder Familie daheim sein %58%; Ausgiebig baden %76%; Auf mich zukommende Situationen in Gedanken bewältigen %45%; </t>
+    <t xml:space="preserve">Mit Partner oder Familie daheim sein %58%; Ausgiebig Tee trinken %76%; Auf mich zukommende Situationen in Gedanken bewältigen %45%; </t>
   </si>
   <si>
     <t>andreas.bröcker@autluuk.kom</t>
@@ -8537,7 +8537,7 @@
     <t>05731 / 79533</t>
   </si>
   <si>
-    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %38%; Mit Arbeitskollegen oder Klassenkameraden sprechen %46%; Eine Blume oder Pflanze sehen oder daran riechen %37%; Eine Dusche nehmen %54%; </t>
+    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %38%; Mit Arbeitskollegen oder Klassenkameraden sprechen %46%; Eine Blume oder Pflanze sehen oder daran riechen %37%; Frische Luft schnappen %54%; </t>
   </si>
   <si>
     <t>kowalski.aleksandra@d-ohnline.kom</t>
@@ -8552,7 +8552,7 @@
     <t>04552 / 98877</t>
   </si>
   <si>
-    <t xml:space="preserve">Mich ärgern, weil ich übervorteilt wurde %89%; Meine Wohnung/Zimmer schön einrichten %16%; Eine Dusche nehmen %26%; </t>
+    <t xml:space="preserve">Mich ärgern, weil ich übervorteilt wurde %89%; Meine Wohnung/Zimmer schön einrichten %16%; Frische Luft schnappen %26%; </t>
   </si>
   <si>
     <t>victoria.schmitz@d-ohnline.kom</t>
@@ -8678,7 +8678,7 @@
     <t>(07331) 8896</t>
   </si>
   <si>
-    <t xml:space="preserve">Dinge in der Natur sammeln (Früchte, Beeren, Steine, usw.) %28%; Videos ansehen %39%; Ausgiebig baden %15%; Positive Zukunftspläne schmieden %71%; </t>
+    <t xml:space="preserve">Dinge in der Natur sammeln (Früchte, Beeren, Steine, usw.) %28%; Videos ansehen %39%; Ausgiebig Tee trinken %15%; Positive Zukunftspläne schmieden %71%; </t>
   </si>
   <si>
     <t>kılıç.türkyılmaz@autluuk.te</t>
@@ -8783,7 +8783,7 @@
     <t>(06130) 93455</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %57%; Post lesen %45%; Für einen guten Zweck spenden %94%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %57%; Post lesen %45%; Für einen guten Zweck spenden %94%; </t>
   </si>
   <si>
     <t>constanze.vogelpohl@gmaiil.ork</t>
@@ -8834,7 +8834,7 @@
     <t>(06261) 7483</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit Arbeitskollegen oder Klassenkameraden sprechen %4%; Einfach abschalten und an nichts denken %88%; Eine Dusche nehmen %38%; </t>
+    <t xml:space="preserve">Mit Arbeitskollegen oder Klassenkameraden sprechen %4%; Einfach abschalten und an nichts denken %88%; Frische Luft schnappen %38%; </t>
   </si>
   <si>
     <t>šimková.marcela@d-ohnline.te</t>
@@ -8897,7 +8897,7 @@
     <t>04341 / 19355</t>
   </si>
   <si>
-    <t xml:space="preserve">Dinge in der Natur sammeln (Früchte, Beeren, Steine, usw.) %18%; Radio hören %85%; Seine Haare waschen %19%; Antiquitäten restaurieren, Möbel aufarbeiten %78%; </t>
+    <t xml:space="preserve">Dinge in der Natur sammeln (Früchte, Beeren, Steine, usw.) %18%; Radio hören %85%; Seine Fotos sortieren %19%; Antiquitäten restaurieren, Möbel aufarbeiten %78%; </t>
   </si>
   <si>
     <t>else.schmelnik@a-o-l.kom</t>
@@ -9059,7 +9059,7 @@
     <t>02953 89175</t>
   </si>
   <si>
-    <t xml:space="preserve">Computer-Netzwerk-Partys %9%; Mit Fremden ins Gespräch kommen %0%; Seine Haare waschen %47%; Eine Dusche nehmen %35%; </t>
+    <t xml:space="preserve">Computer-Netzwerk-Partys %9%; Mit Fremden ins Gespräch kommen %0%; Seine Fotos sortieren %47%; Frische Luft schnappen %35%; </t>
   </si>
   <si>
     <t>eva.hahn@a-o-l.ork</t>
@@ -9392,7 +9392,7 @@
     <t>0168 / 143067</t>
   </si>
   <si>
-    <t xml:space="preserve">Einfach alleine sein %52%; Eine Dusche nehmen %31%; </t>
+    <t xml:space="preserve">Einfach alleine sein %52%; Frische Luft schnappen %31%; </t>
   </si>
   <si>
     <t>dirk.beitelhoff@autluuk.te</t>
@@ -9767,7 +9767,7 @@
     <t>(04195) 87312</t>
   </si>
   <si>
-    <t xml:space="preserve">Etwas neuartig und originell machen %46%; Kochen oder backen %0%; Eine Dusche nehmen %14%; </t>
+    <t xml:space="preserve">Etwas neuartig und originell machen %46%; Kochen oder backen %0%; Frische Luft schnappen %14%; </t>
   </si>
   <si>
     <t>werner.rohm@autluuk.te</t>
@@ -9824,7 +9824,7 @@
     <t>0354 / 524941</t>
   </si>
   <si>
-    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %54%; Etwas Neues lernen %41%; Ausgiebig frühstücken %7%; Eine Dusche nehmen %6%; </t>
+    <t xml:space="preserve">Kegeln oder einen Gymnastikkurs besuchen %54%; Etwas Neues lernen %41%; Ausgiebig frühstücken %7%; Frische Luft schnappen %6%; </t>
   </si>
   <si>
     <t>detlef.kecker@gmaiil.te</t>
@@ -10193,7 +10193,7 @@
     <t>05208 / 56761</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine schwierige Aufgabe meistern %45%; Ausgiebig baden %91%; Ausschlafen %51%; </t>
+    <t xml:space="preserve">Eine schwierige Aufgabe meistern %45%; Ausgiebig Tee trinken %91%; Ausschlafen %51%; </t>
   </si>
   <si>
     <t>sylvia.micklich@gmaiil.te</t>
@@ -10703,7 +10703,7 @@
     <t>(05427) 58700</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgiebig baden %7%; Antiquitäten restaurieren, Möbel aufarbeiten %87%; </t>
+    <t xml:space="preserve">Ausgiebig Tee trinken %7%; Antiquitäten restaurieren, Möbel aufarbeiten %87%; </t>
   </si>
   <si>
     <t>jörg.patrzek@a-o-l.te</t>
@@ -10733,7 +10733,7 @@
     <t>03661 / 87670</t>
   </si>
   <si>
-    <t xml:space="preserve">In einem Café sitzen %35%; Ins Kino gehen %4%; Mit Freunden oder Bekannten zusammen essen %92%; Ausgiebig baden %11%; Ein Nickerchen machen %49%; </t>
+    <t xml:space="preserve">In einem Café sitzen %35%; Ins Kino gehen %4%; Mit Freunden oder Bekannten zusammen essen %92%; Ausgiebig Tee trinken %11%; Ein Nickerchen machen %49%; </t>
   </si>
   <si>
     <t>franz.konrad@autluuk.te</t>
@@ -10970,7 +10970,7 @@
     <t>09471 / 89611</t>
   </si>
   <si>
-    <t xml:space="preserve">Fremdsprachenkenntnisse erweitern %57%; Zärtlich sein, schmusen, küssen %97%; Einfach mit guten Freunden zwanglos plaudern %58%; Ein Nickerchen machen %57%; </t>
+    <t xml:space="preserve">Fremdsprachenkenntnisse erweitern %57%; Einen gemütlichen Filmabend machen %97%; Einfach mit guten Freunden zwanglos plaudern %58%; Ein Nickerchen machen %57%; </t>
   </si>
   <si>
     <t>blažková.marta@gmaiil.te</t>
@@ -11162,7 +11162,7 @@
     <t>050 / 8345564</t>
   </si>
   <si>
-    <t xml:space="preserve">Etwas Neues lernen %81%; Gegenstände reparieren %94%; Eine Dusche nehmen %21%; </t>
+    <t xml:space="preserve">Etwas Neues lernen %81%; Gegenstände reparieren %94%; Frische Luft schnappen %21%; </t>
   </si>
   <si>
     <t>nina.maibaum@web.te</t>
@@ -11177,7 +11177,7 @@
     <t>0160 / 872732</t>
   </si>
   <si>
-    <t xml:space="preserve">An einer Tagung teilnehmen %5%; Witze anhören %96%; Möglichst pünktlich wegkommen %18%; Fachliteratur oder Sachbuch lesen %99%; Eine Dusche nehmen %24%; </t>
+    <t xml:space="preserve">An einer Tagung teilnehmen %5%; Witze anhören %96%; Möglichst pünktlich wegkommen %18%; Fachliteratur oder Sachbuch lesen %99%; Frische Luft schnappen %24%; </t>
   </si>
   <si>
     <t>markus.angeli@gmaiil.ork</t>
@@ -11342,7 +11342,7 @@
     <t>04151 60186</t>
   </si>
   <si>
-    <t xml:space="preserve">Alte Freunde wieder treffen %9%; Etwas schmackhaftes zu mir nehmen %22%; Eine Dusche nehmen %36%; </t>
+    <t xml:space="preserve">Alte Freunde wieder treffen %9%; Etwas schmackhaftes zu mir nehmen %22%; Frische Luft schnappen %36%; </t>
   </si>
   <si>
     <t>25.11.1970</t>
@@ -11369,7 +11369,7 @@
     <t>(0451) 770201</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %65%; Etwas neuartig und originell machen %43%; Mir selbst etwas kochen %85%; Für einen guten Zweck spenden %5%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %65%; Etwas neuartig und originell machen %43%; Mir selbst etwas kochen %85%; Für einen guten Zweck spenden %5%; </t>
   </si>
   <si>
     <t>friedhelm.schmitte@gmaiil.ork</t>
@@ -12164,7 +12164,7 @@
     <t>(0631) 511474</t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %65%; Kochen oder backen %48%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %65%; Kochen oder backen %48%; </t>
   </si>
   <si>
     <t>bytyqi.adem@d-ohnline.te</t>
@@ -12179,7 +12179,7 @@
     <t>(07662) 90380</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit seinem Partner zusammen sein %84%; Briefe an Verwandte und Bekannte schreiben %62%; Eine Dusche nehmen %71%; </t>
+    <t xml:space="preserve">Mit seinem Partner zusammen sein %84%; Briefe an Verwandte und Bekannte schreiben %62%; Frische Luft schnappen %71%; </t>
   </si>
   <si>
     <t>katrin.timmer@autluuk.te</t>
@@ -12260,7 +12260,7 @@
     <t>08341 / 88849</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine Dusche nehmen %1%; </t>
+    <t xml:space="preserve">Frische Luft schnappen %1%; </t>
   </si>
   <si>
     <t>nowak.piotr@web.ork</t>
@@ -12413,7 +12413,7 @@
     <t>0991 / 428516</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich mit Tieren beschäftigen %47%; Jemandem helfen %75%; Seine Haare waschen %86%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %51%; </t>
+    <t xml:space="preserve">Sich mit Tieren beschäftigen %47%; Jemandem helfen %75%; Seine Fotos sortieren %86%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %51%; </t>
   </si>
   <si>
     <t>delić.milorad@autluuk.te</t>
@@ -12443,7 +12443,7 @@
     <t>(04336) 47560</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %79%; Möglichst pünktlich wegkommen %94%; Für einen guten Zweck spenden %91%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %79%; Möglichst pünktlich wegkommen %94%; Für einen guten Zweck spenden %91%; </t>
   </si>
   <si>
     <t>12.10.1981</t>
@@ -12851,7 +12851,7 @@
     <t>(038205) 1427</t>
   </si>
   <si>
-    <t xml:space="preserve">Wasserski laufen, surfen, tauchen %87%; Zärtlich sein, schmusen, küssen %13%; Morgens Früh aufstehen %87%; Etwas planen oder organisieren %44%; </t>
+    <t xml:space="preserve">Wasserski laufen, surfen, tauchen %87%; Einen gemütlichen Filmabend machen %13%; Morgens Früh aufstehen %87%; Etwas planen oder organisieren %44%; </t>
   </si>
   <si>
     <t>willi.krone@gmaiil.te</t>
@@ -12881,7 +12881,7 @@
     <t>030 / 8058686</t>
   </si>
   <si>
-    <t xml:space="preserve">Malen, basteln, musizieren, usw. %69%; Eine Dusche nehmen %57%; </t>
+    <t xml:space="preserve">Malen, basteln, musizieren, usw. %69%; Frische Luft schnappen %57%; </t>
   </si>
   <si>
     <t>tobias.husmeier@iunitimail.te</t>
@@ -12941,7 +12941,7 @@
     <t>(05431) 819</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %23%; Eine schwierige Aufgabe meistern %25%; Faulenzen %94%; Etwas lernen und mich fortbilden %12%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %23%; Eine schwierige Aufgabe meistern %25%; Faulenzen %94%; Etwas lernen und mich fortbilden %12%; </t>
   </si>
   <si>
     <t>gita.päts@d-ohnline.te</t>
@@ -12956,7 +12956,7 @@
     <t>(0235) 836059</t>
   </si>
   <si>
-    <t xml:space="preserve">Ins Kino gehen %55%; Über meine Arbeit reden %96%; Ausgiebig baden %80%; </t>
+    <t xml:space="preserve">Ins Kino gehen %55%; Über meine Arbeit reden %96%; Ausgiebig Tee trinken %80%; </t>
   </si>
   <si>
     <t>thomas.fischer@d-ohnline.ork</t>
@@ -13064,7 +13064,7 @@
     <t>06071 / 90268</t>
   </si>
   <si>
-    <t xml:space="preserve">In ein Lokal gehen %94%; Mit meiner Meinung Recht haben %65%; Cartoons, Comic-Hefte lesen %68%; Eine Dusche nehmen %49%; </t>
+    <t xml:space="preserve">In ein Lokal gehen %94%; Mit meiner Meinung Recht haben %65%; Cartoons, Comic-Hefte lesen %68%; Frische Luft schnappen %49%; </t>
   </si>
   <si>
     <t>ostrowski.zbigniew@autluuk.ork</t>
@@ -13097,7 +13097,7 @@
     <t>02077 / 64221</t>
   </si>
   <si>
-    <t xml:space="preserve">Holz hacken %3%; Mein Recht durchsetzen und andere zum Nachgeben bewegen %21%; Kreuzworträtsel lösen oder ein Puzzle legen %80%; Eine Dusche nehmen %92%; </t>
+    <t xml:space="preserve">Holz hacken %3%; Mein Recht durchsetzen und andere zum Nachgeben bewegen %21%; Kreuzworträtsel lösen oder ein Puzzle legen %80%; Frische Luft schnappen %92%; </t>
   </si>
   <si>
     <t>wolfgang.böttger@gmaiil.te</t>
@@ -13184,7 +13184,7 @@
     <t>(0531) 381729</t>
   </si>
   <si>
-    <t xml:space="preserve">Etwas zügig erledigen %74%; Cartoons, Comic-Hefte lesen %93%; Eine Dusche nehmen %34%; </t>
+    <t xml:space="preserve">Etwas zügig erledigen %74%; Cartoons, Comic-Hefte lesen %93%; Frische Luft schnappen %34%; </t>
   </si>
   <si>
     <t>bruno.neher@ge-em-ix.ork</t>
@@ -13214,7 +13214,7 @@
     <t>06224 / 38868</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %80%; Ein Nickerchen machen %45%; </t>
+    <t xml:space="preserve">Für jemanden kochen %80%; Ein Nickerchen machen %45%; </t>
   </si>
   <si>
     <t>markus.walbaum@autluuk.ork</t>
@@ -13229,7 +13229,7 @@
     <t>(04331) 30353</t>
   </si>
   <si>
-    <t xml:space="preserve">Gäste einladen %18%; Jemanden massieren %33%; Etwas fertig stellen %63%; Faulenzen %17%; Leger gekleidet sein %61%; </t>
+    <t xml:space="preserve">Gäste einladen %18%; Für jemanden kochen %33%; Etwas fertig stellen %63%; Faulenzen %17%; Leger gekleidet sein %61%; </t>
   </si>
   <si>
     <t>ursula.schilling@ge-em-ix.ork</t>
@@ -13394,7 +13394,7 @@
     <t>02653 / 84770</t>
   </si>
   <si>
-    <t xml:space="preserve">Über sein Hobby oder spezielles Interessengebiet reden %16%; Ausgiebig baden %53%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %99%; </t>
+    <t xml:space="preserve">Über sein Hobby oder spezielles Interessengebiet reden %16%; Ausgiebig Tee trinken %53%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %99%; </t>
   </si>
   <si>
     <t>raimund.hach@autluuk.te</t>
@@ -13472,7 +13472,7 @@
     <t>02181 / 35580</t>
   </si>
   <si>
-    <t xml:space="preserve">Radio hören %40%; Kreuzworträtsel lösen oder ein Puzzle legen %16%; Eine Dusche nehmen %95%; </t>
+    <t xml:space="preserve">Radio hören %40%; Kreuzworträtsel lösen oder ein Puzzle legen %16%; Frische Luft schnappen %95%; </t>
   </si>
   <si>
     <t>leopold.dierkes@ge-em-ix.te</t>
@@ -13565,7 +13565,7 @@
     <t>(0168) 125279</t>
   </si>
   <si>
-    <t xml:space="preserve">Ringen oder boxen %26%; Zärtlich sein, schmusen, küssen %77%; Sich um neue Arbeit bewerben %58%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %59%; </t>
+    <t xml:space="preserve">Ringen oder boxen %26%; Einen gemütlichen Filmabend machen %77%; Sich um neue Arbeit bewerben %58%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %59%; </t>
   </si>
   <si>
     <t>carolin.belau@ge-em-ix.te</t>
@@ -13658,7 +13658,7 @@
     <t>07125 / 8047</t>
   </si>
   <si>
-    <t xml:space="preserve">Schwierige Probleme klären %8%; Seine Haare waschen %55%; Private Sachen erledigen, die schon lange liegengeblieben sind %13%; </t>
+    <t xml:space="preserve">Schwierige Probleme klären %8%; Seine Fotos sortieren %55%; Private Sachen erledigen, die schon lange liegengeblieben sind %13%; </t>
   </si>
   <si>
     <t>klaus.sender@d-ohnline.te</t>
@@ -13811,7 +13811,7 @@
     <t>02425 / 83677</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %22%; Radio hören %77%; Positive Zukunftspläne schmieden %46%; </t>
+    <t xml:space="preserve">Für jemanden kochen %22%; Radio hören %77%; Positive Zukunftspläne schmieden %46%; </t>
   </si>
   <si>
     <t>hermann.glanemann@gmaiil.te</t>
@@ -13979,7 +13979,7 @@
     <t>05231 / 6316</t>
   </si>
   <si>
-    <t xml:space="preserve">Kartenspielen %23%; Mich laut beschweren %12%; Ausgiebig baden %16%; Etwas entwerfen oder zeichnen %73%; </t>
+    <t xml:space="preserve">Kartenspielen %23%; Mich laut beschweren %12%; Ausgiebig Tee trinken %16%; Etwas entwerfen oder zeichnen %73%; </t>
   </si>
   <si>
     <t>martin.müller@iunitimail.kom</t>
@@ -14153,7 +14153,7 @@
     <t>07662 85053</t>
   </si>
   <si>
-    <t xml:space="preserve">Holz hacken %2%; Landkarten studieren %98%; Seine finanziellen Angelegenheiten regeln %22%; Eine Dusche nehmen %64%; </t>
+    <t xml:space="preserve">Holz hacken %2%; Landkarten studieren %98%; Seine finanziellen Angelegenheiten regeln %22%; Frische Luft schnappen %64%; </t>
   </si>
   <si>
     <t>heike.tietjen@iunitimail.kom</t>
@@ -14636,7 +14636,7 @@
     <t>0411 / 309791</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit Partner oder Familie daheim sein %31%; Eine Dusche nehmen %53%; </t>
+    <t xml:space="preserve">Mit Partner oder Familie daheim sein %31%; Frische Luft schnappen %53%; </t>
   </si>
   <si>
     <t>wolfgang.quoss@web.kom</t>
@@ -15320,7 +15320,7 @@
     <t>07732 / 55152</t>
   </si>
   <si>
-    <t xml:space="preserve">Seine Haare waschen %74%; </t>
+    <t xml:space="preserve">Seine Fotos sortieren %74%; </t>
   </si>
   <si>
     <t>dominguez.nuria@autluuk.kom</t>
@@ -15512,7 +15512,7 @@
     <t>06101 / 6935</t>
   </si>
   <si>
-    <t xml:space="preserve">Über meine Probleme reden %80%; Seine Haare waschen %83%; Eine Dusche nehmen %0%; </t>
+    <t xml:space="preserve">Über meine Probleme reden %80%; Seine Fotos sortieren %83%; Frische Luft schnappen %0%; </t>
   </si>
   <si>
     <t>hamoud.mariam@gmaiil.te</t>
@@ -15881,7 +15881,7 @@
     <t>06051 / 49985</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine Sache klipp und klar sagen %91%; Seine Haare waschen %39%; Ausschlafen %85%; </t>
+    <t xml:space="preserve">Eine Sache klipp und klar sagen %91%; Seine Fotos sortieren %39%; Ausschlafen %85%; </t>
   </si>
   <si>
     <t>navarro.lucia@gmaiil.kom</t>
@@ -15911,7 +15911,7 @@
     <t>07924 / 30535</t>
   </si>
   <si>
-    <t xml:space="preserve">An einem sportlichen Wettbewerb teilnehmen %33%; Möglichst pünktlich wegkommen %88%; Ausgiebig baden %42%; Positive Zukunftspläne schmieden %61%; </t>
+    <t xml:space="preserve">An einem sportlichen Wettbewerb teilnehmen %33%; Möglichst pünktlich wegkommen %88%; Ausgiebig Tee trinken %42%; Positive Zukunftspläne schmieden %61%; </t>
   </si>
   <si>
     <t>jan.topyürek@ge-em-ix.ork</t>
@@ -16043,7 +16043,7 @@
     <t>05182 / 82467</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich politisch oder sozial betätigen %62%; Andere Leute betrachten %33%; Musik hören %74%; Eine Dusche nehmen %16%; </t>
+    <t xml:space="preserve">Sich politisch oder sozial betätigen %62%; Andere Leute betrachten %33%; Musik hören %74%; Frische Luft schnappen %16%; </t>
   </si>
   <si>
     <t>willy.meyer@gmaiil.te</t>
@@ -16307,7 +16307,7 @@
     <t>07163 / 47219</t>
   </si>
   <si>
-    <t xml:space="preserve">Gymnastik, Fitnessübungen betreiben %98%; Jemanden massieren %33%; Einfach alleine sein %66%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %62%; </t>
+    <t xml:space="preserve">Gymnastik, Fitnessübungen betreiben %98%; Für jemanden kochen %33%; Einfach alleine sein %66%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %62%; </t>
   </si>
   <si>
     <t>michael.sons@ge-em-ix.ork</t>
@@ -16373,7 +16373,7 @@
     <t>02302 / 26240</t>
   </si>
   <si>
-    <t xml:space="preserve">Billard spielen %61%; Den Himmel, Wolken oder einen breiten Sturm beobachten %76%; Ausgiebig baden %7%; Auf mich zukommende Situationen in Gedanken bewältigen %9%; </t>
+    <t xml:space="preserve">Billard spielen %61%; Den Himmel, Wolken oder einen breiten Sturm beobachten %76%; Ausgiebig Tee trinken %7%; Auf mich zukommende Situationen in Gedanken bewältigen %9%; </t>
   </si>
   <si>
     <t>virginia.elich@d-ohnline.ork</t>
@@ -16724,7 +16724,7 @@
     <t>05131 / 42023</t>
   </si>
   <si>
-    <t xml:space="preserve">Wandern %95%; Etwas zügig erledigen %85%; Eine Dusche nehmen %68%; </t>
+    <t xml:space="preserve">Wandern %95%; Etwas zügig erledigen %85%; Frische Luft schnappen %68%; </t>
   </si>
   <si>
     <t>manfred.melchers@web.kom</t>
@@ -16865,7 +16865,7 @@
     <t>06192 / 2333</t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %93%; Mit Arbeitskollegen oder Klassenkameraden sprechen %5%; Fotos oder Dias anschauen %21%; Ein Nickerchen machen %1%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %93%; Mit Arbeitskollegen oder Klassenkameraden sprechen %5%; Fotos oder Dias anschauen %21%; Ein Nickerchen machen %1%; </t>
   </si>
   <si>
     <t>shevchenko.vadim@1mal1.kom</t>
@@ -17066,7 +17066,7 @@
     <t>(02043) 58637</t>
   </si>
   <si>
-    <t xml:space="preserve">Erkundungsgänge machen (unbekannte Gegenden) %4%; Ein Konzert, eine Opern- oder Ballettaufführung besuchen %29%; Mit einer Spielekonsole spielen %35%; Seine Haare waschen %26%; </t>
+    <t xml:space="preserve">Erkundungsgänge machen (unbekannte Gegenden) %4%; Ein Konzert, eine Opern- oder Ballettaufführung besuchen %29%; Mit einer Spielekonsole spielen %35%; Seine Fotos sortieren %26%; </t>
   </si>
   <si>
     <t>rusu.raluca@iunitimail.te</t>
@@ -17081,7 +17081,7 @@
     <t>(0162) 261926</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %92%; Jemandem eine Freude bereiten %81%; Tagträumen %47%; Antiquitäten restaurieren, Möbel aufarbeiten %98%; </t>
+    <t xml:space="preserve">Für jemanden kochen %92%; Jemandem eine Freude bereiten %81%; Tagträumen %47%; Antiquitäten restaurieren, Möbel aufarbeiten %98%; </t>
   </si>
   <si>
     <t>uwe.banach@gmaiil.te</t>
@@ -17360,7 +17360,7 @@
     <t>0162 / 452267</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %27%; Etwas zügig erledigen %50%; Parfum benutzen %70%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %27%; Etwas zügig erledigen %50%; Parfum benutzen %70%; </t>
   </si>
   <si>
     <t>claudia.bartz@1mal1.ork</t>
@@ -17720,7 +17720,7 @@
     <t>02342 / 12958</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %88%; Eine Blume oder Pflanze sehen oder daran riechen %62%; An meine Freunde und Bekannten denken %96%; </t>
+    <t xml:space="preserve">Für jemanden kochen %88%; Eine Blume oder Pflanze sehen oder daran riechen %62%; An meine Freunde und Bekannten denken %96%; </t>
   </si>
   <si>
     <t>annalouise.foitzik@iunitimail.kom</t>
@@ -17735,7 +17735,7 @@
     <t>05425 14285</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %16%; Mit meiner Meinung Recht haben %19%; Sich entspannen %30%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %16%; Mit meiner Meinung Recht haben %19%; Sich entspannen %30%; </t>
   </si>
   <si>
     <t>28.01.1979</t>
@@ -17858,7 +17858,7 @@
     <t>02074 / 3714</t>
   </si>
   <si>
-    <t xml:space="preserve">Entspannungsübungen machen %71%; Eine Dusche nehmen %96%; </t>
+    <t xml:space="preserve">Entspannungsübungen machen %71%; Frische Luft schnappen %96%; </t>
   </si>
   <si>
     <t>horst.boskovich@a-o-l.te</t>
@@ -17948,7 +17948,7 @@
     <t>0931 / 918675</t>
   </si>
   <si>
-    <t xml:space="preserve">Reiten %21%; Jemanden massieren %86%; Videos ansehen %29%; Einen Spaziergang machen %9%; Positive Zukunftspläne schmieden %11%; </t>
+    <t xml:space="preserve">Reiten %21%; Für jemanden kochen %86%; Videos ansehen %29%; Einen Spaziergang machen %9%; Positive Zukunftspläne schmieden %11%; </t>
   </si>
   <si>
     <t>xíngjiàn.fāng@gmaiil.te</t>
@@ -17966,7 +17966,7 @@
     <t>(06331) 75716</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %9%; Sich über Sport unterhalten %72%; Tagträumen %29%; Etwas lernen und mich fortbilden %17%; </t>
+    <t xml:space="preserve">Für jemanden kochen %9%; Sich über Sport unterhalten %72%; Tagträumen %29%; Etwas lernen und mich fortbilden %17%; </t>
   </si>
   <si>
     <t>piotrowski.alicja@d-ohnline.te</t>
@@ -18086,7 +18086,7 @@
     <t>07165 / 95192</t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %78%; Um Hilfe und Ratschläge bitten %10%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %78%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %78%; Um Hilfe und Ratschläge bitten %10%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %78%; </t>
   </si>
   <si>
     <t>volker.souseribeirodomingues@d-ohnline.te</t>
@@ -18566,7 +18566,7 @@
     <t>0551 / 821590</t>
   </si>
   <si>
-    <t xml:space="preserve">Auf Volksfeste gehen %97%; Streit aus dem Wege gehen %18%; Seine Haare waschen %94%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %24%; </t>
+    <t xml:space="preserve">Auf Volksfeste gehen %97%; Streit aus dem Wege gehen %18%; Seine Fotos sortieren %94%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %24%; </t>
   </si>
   <si>
     <t>michael.nischk@gmaiil.ork</t>
@@ -18581,7 +18581,7 @@
     <t>050 6471141</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %16%; Mit Fremden ins Gespräch kommen %69%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %16%; Mit Fremden ins Gespräch kommen %69%; </t>
   </si>
   <si>
     <t>michaela.lorbach@a-o-l.te</t>
@@ -18659,7 +18659,7 @@
     <t>(05202) 13335</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %41%; Für andere sorgen %10%; Tagebuch schreiben %86%; Etwas planen oder organisieren %44%; </t>
+    <t xml:space="preserve">Für jemanden kochen %41%; Für andere sorgen %10%; Tagebuch schreiben %86%; Etwas planen oder organisieren %44%; </t>
   </si>
   <si>
     <t>frank.meyerhoff@a-o-l.kom</t>
@@ -19055,7 +19055,7 @@
     <t>05122 / 71742</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine Dusche nehmen %58%; </t>
+    <t xml:space="preserve">Frische Luft schnappen %58%; </t>
   </si>
   <si>
     <t>ernst.meier@1mal1.ork</t>
@@ -19070,7 +19070,7 @@
     <t>033203 / 6768</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %2%; Tagebuch schreiben %57%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %84%; </t>
+    <t xml:space="preserve">Für jemanden kochen %2%; Tagebuch schreiben %57%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %84%; </t>
   </si>
   <si>
     <t>bernt.jakobtorweihe@a-o-l.te</t>
@@ -19106,7 +19106,7 @@
     <t>02572 / 35239</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgiebig frühstücken %4%; Eine Dusche nehmen %39%; </t>
+    <t xml:space="preserve">Ausgiebig frühstücken %4%; Frische Luft schnappen %39%; </t>
   </si>
   <si>
     <t>taylor.jennifer@gmaiil.ork</t>
@@ -19250,7 +19250,7 @@
     <t>(09131) 2822</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine Blume oder Pflanze sehen oder daran riechen %35%; Eine Dusche nehmen %58%; </t>
+    <t xml:space="preserve">Eine Blume oder Pflanze sehen oder daran riechen %35%; Frische Luft schnappen %58%; </t>
   </si>
   <si>
     <t>karim.yunis@autluuk.kom</t>
@@ -19733,7 +19733,7 @@
     <t>02181 / 49830</t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %43%; Über meine Probleme reden %95%; Einfach alleine sein %67%; Etwas planen oder organisieren %70%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %43%; Über meine Probleme reden %95%; Einfach alleine sein %67%; Etwas planen oder organisieren %70%; </t>
   </si>
   <si>
     <t>matthias.diekmann@iunitimail.te</t>
@@ -19793,7 +19793,7 @@
     <t>02392 21598</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden beraten %13%; Radio hören %53%; Einfach alleine sein %62%; Eine Dusche nehmen %24%; </t>
+    <t xml:space="preserve">Jemanden beraten %13%; Radio hören %53%; Einfach alleine sein %62%; Frische Luft schnappen %24%; </t>
   </si>
   <si>
     <t>kai.füchtenbusch@1mal1.kom</t>
@@ -19883,7 +19883,7 @@
     <t>(02261) 39037</t>
   </si>
   <si>
-    <t xml:space="preserve">Neue Bekanntschaften machen %6%; Cartoons, Comic-Hefte lesen %67%; Eine Dusche nehmen %95%; </t>
+    <t xml:space="preserve">Neue Bekanntschaften machen %6%; Cartoons, Comic-Hefte lesen %67%; Frische Luft schnappen %95%; </t>
   </si>
   <si>
     <t>claudia.effing@d-ohnline.kom</t>
@@ -19985,7 +19985,7 @@
     <t>078 5735393</t>
   </si>
   <si>
-    <t xml:space="preserve">Wasserski laufen, surfen, tauchen %38%; Jemanden massieren %11%; Im Internet surfen %98%; Eine Anschaffung machen (Auto, Hausgegenstände, etc.) %86%; Private Sachen erledigen, die schon lange liegengeblieben sind %24%; </t>
+    <t xml:space="preserve">Wasserski laufen, surfen, tauchen %38%; Für jemanden kochen %11%; Im Internet surfen %98%; Eine Anschaffung machen (Auto, Hausgegenstände, etc.) %86%; Private Sachen erledigen, die schon lange liegengeblieben sind %24%; </t>
   </si>
   <si>
     <t>markus.trost@1mal1.kom</t>
@@ -20159,7 +20159,7 @@
     <t>04221 / 10204</t>
   </si>
   <si>
-    <t xml:space="preserve">Neue Leute kennen lernen %94%; Seine Haare waschen %79%; Etwas planen oder organisieren %7%; </t>
+    <t xml:space="preserve">Neue Leute kennen lernen %94%; Seine Fotos sortieren %79%; Etwas planen oder organisieren %7%; </t>
   </si>
   <si>
     <t>rudolf.rüdiger@ge-em-ix.te</t>
@@ -20444,7 +20444,7 @@
     <t>02325 / 44960</t>
   </si>
   <si>
-    <t xml:space="preserve">Landkarten studieren %42%; Eine Dusche nehmen %70%; </t>
+    <t xml:space="preserve">Landkarten studieren %42%; Frische Luft schnappen %70%; </t>
   </si>
   <si>
     <t>catharina.fehl@web.ork</t>
@@ -20459,7 +20459,7 @@
     <t>06041 / 36329</t>
   </si>
   <si>
-    <t xml:space="preserve">Neue Bekanntschaften machen %89%; Seine Haare waschen %22%; </t>
+    <t xml:space="preserve">Neue Bekanntschaften machen %89%; Seine Fotos sortieren %22%; </t>
   </si>
   <si>
     <t>albert.vandeloo@gmaiil.te</t>
@@ -20537,7 +20537,7 @@
     <t>06091 / 18238</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %59%; Am Ofen/Kamin sitzen, ins Feuer gucken %94%; Etwas lernen und mich fortbilden %93%; </t>
+    <t xml:space="preserve">Für jemanden kochen %59%; Am Ofen/Kamin sitzen, ins Feuer gucken %94%; Etwas lernen und mich fortbilden %93%; </t>
   </si>
   <si>
     <t>astrid.vassmer@autluuk.te</t>
@@ -20672,7 +20672,7 @@
     <t>02065 / 86816</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgiebig baden %20%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %10%; </t>
+    <t xml:space="preserve">Ausgiebig Tee trinken %20%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %10%; </t>
   </si>
   <si>
     <t>acar.nehir@ge-em-ix.kom</t>
@@ -20720,7 +20720,7 @@
     <t>06821 / 30869</t>
   </si>
   <si>
-    <t xml:space="preserve">Sport treiben %85%; Blog im Internet schreiben %88%; Zeitung lesen %91%; Eine Dusche nehmen %5%; </t>
+    <t xml:space="preserve">Sport treiben %85%; Blog im Internet schreiben %88%; Zeitung lesen %91%; Frische Luft schnappen %5%; </t>
   </si>
   <si>
     <t>bajrami.violeta@gmaiil.kom</t>
@@ -20789,7 +20789,7 @@
     <t>05821 / 1561</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgiebig baden %43%; An technischen Dingen arbeiten (Fahrzeuge, Hausgeräte usw.) %0%; </t>
+    <t xml:space="preserve">Ausgiebig Tee trinken %43%; An technischen Dingen arbeiten (Fahrzeuge, Hausgeräte usw.) %0%; </t>
   </si>
   <si>
     <t>06.09.1988</t>
@@ -20936,7 +20936,7 @@
     <t>0160 / 542471</t>
   </si>
   <si>
-    <t xml:space="preserve">Im Wasser waten %70%; Computerspiele spielen %52%; Sich um Zimmerpflanzen kümmern %29%; Eine Dusche nehmen %96%; </t>
+    <t xml:space="preserve">Im Wasser waten %70%; Computerspiele spielen %52%; Sich um Zimmerpflanzen kümmern %29%; Frische Luft schnappen %96%; </t>
   </si>
   <si>
     <t>jan.andersson@gmaiil.te</t>
@@ -20978,7 +20978,7 @@
     <t>0391 / 602662</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %18%; Private Sachen erledigen, die schon lange liegengeblieben sind %34%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %18%; Private Sachen erledigen, die schon lange liegengeblieben sind %34%; </t>
   </si>
   <si>
     <t>hans-gregor.koops@1mal1.kom</t>
@@ -20993,7 +20993,7 @@
     <t>0461 / 971420</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit Fremden ins Gespräch kommen %53%; Faulenzen %66%; Eine Dusche nehmen %58%; </t>
+    <t xml:space="preserve">Mit Fremden ins Gespräch kommen %53%; Faulenzen %66%; Frische Luft schnappen %58%; </t>
   </si>
   <si>
     <t>simone.schulte@gmaiil.ork</t>
@@ -21080,7 +21080,7 @@
     <t>050 / 7448729</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine schwierige Aufgabe meistern %11%; Seine Haare waschen %95%; Etwas lernen und mich fortbilden %43%; </t>
+    <t xml:space="preserve">Eine schwierige Aufgabe meistern %11%; Seine Fotos sortieren %95%; Etwas lernen und mich fortbilden %43%; </t>
   </si>
   <si>
     <t>anja.mallek@autluuk.ork</t>
@@ -21158,7 +21158,7 @@
     <t>02563 / 93903</t>
   </si>
   <si>
-    <t xml:space="preserve">Tennis spielen %93%; Jemandem behilflich sein %35%; Am Ofen/Kamin sitzen, ins Feuer gucken %63%; Eine Dusche nehmen %43%; </t>
+    <t xml:space="preserve">Tennis spielen %93%; Jemandem behilflich sein %35%; Am Ofen/Kamin sitzen, ins Feuer gucken %63%; Frische Luft schnappen %43%; </t>
   </si>
   <si>
     <t>tobias.gerhard@gmaiil.te</t>
@@ -21287,7 +21287,7 @@
     <t>07321 / 24357</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden telefonisch zu einem Treffen einladen %85%; Über meine Interessen diskutieren %67%; Blumen kaufen %63%; Eine Dusche nehmen %0%; </t>
+    <t xml:space="preserve">Jemanden telefonisch zu einem Treffen einladen %85%; Über meine Interessen diskutieren %67%; Blumen kaufen %63%; Frische Luft schnappen %0%; </t>
   </si>
   <si>
     <t>kaczmarek.karol@1mal1.kom</t>
@@ -21374,7 +21374,7 @@
     <t>030 / 4496015</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgiebig baden %7%; Etwas lernen und mich fortbilden %66%; </t>
+    <t xml:space="preserve">Ausgiebig Tee trinken %7%; Etwas lernen und mich fortbilden %66%; </t>
   </si>
   <si>
     <t>elisabeth.hermes@d-ohnline.te</t>
@@ -21821,7 +21821,7 @@
     <t>050 / 1134360</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden beraten %85%; Kräuter/Pilze sammeln %36%; Eine Dusche nehmen %33%; </t>
+    <t xml:space="preserve">Jemanden beraten %85%; Kräuter/Pilze sammeln %36%; Frische Luft schnappen %33%; </t>
   </si>
   <si>
     <t>marcus.linneweber@a-o-l.te</t>
@@ -21881,7 +21881,7 @@
     <t>0371 973596</t>
   </si>
   <si>
-    <t xml:space="preserve">Ins Theater gehen %72%; Sport treiben %51%; Mir selbst etwas kochen %34%; Eine Dusche nehmen %28%; </t>
+    <t xml:space="preserve">Ins Theater gehen %72%; Sport treiben %51%; Mir selbst etwas kochen %34%; Frische Luft schnappen %28%; </t>
   </si>
   <si>
     <t>karola.klingel@gmaiil.kom</t>
@@ -21962,7 +21962,7 @@
     <t>(04141) 11141</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %70%; Seine finanziellen Angelegenheiten regeln %49%; Eine Dusche nehmen %72%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %70%; Seine finanziellen Angelegenheiten regeln %49%; Frische Luft schnappen %72%; </t>
   </si>
   <si>
     <t>martin.riegel@web.ork</t>
@@ -21995,7 +21995,7 @@
     <t>(04351) 66339</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %3%; Mit Freunden oder Bekannten zusammen essen %6%; An meine Freunde und Bekannten denken %31%; </t>
+    <t xml:space="preserve">Für jemanden kochen %3%; Mit Freunden oder Bekannten zusammen essen %6%; An meine Freunde und Bekannten denken %31%; </t>
   </si>
   <si>
     <t>johannes.schlüter@d-ohnline.te</t>
@@ -22067,7 +22067,7 @@
     <t>02045 / 77675</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %11%; Ausschlafen %17%; </t>
+    <t xml:space="preserve">Für jemanden kochen %11%; Ausschlafen %17%; </t>
   </si>
   <si>
     <t>henril..borchert@web.te</t>
@@ -22244,7 +22244,7 @@
     <t>(030) 3914032</t>
   </si>
   <si>
-    <t xml:space="preserve">Andere Leute betrachten %24%; Einfach abschalten und an nichts denken %76%; Eine Dusche nehmen %35%; </t>
+    <t xml:space="preserve">Andere Leute betrachten %24%; Einfach abschalten und an nichts denken %76%; Frische Luft schnappen %35%; </t>
   </si>
   <si>
     <t>nellya..hürter@gmaiil.te</t>
@@ -22400,7 +22400,7 @@
     <t>0831 / 597574</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit Freunden zusammen sein %65%; Einen Spaziergang machen %98%; Eine Dusche nehmen %28%; </t>
+    <t xml:space="preserve">Mit Freunden zusammen sein %65%; Einen Spaziergang machen %98%; Frische Luft schnappen %28%; </t>
   </si>
   <si>
     <t>hedwig.wydra@web.te</t>
@@ -22523,7 +22523,7 @@
     <t>04131 / 29271</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %27%; Mich vor dem Spiegel zurechtmachen %42%; Mich meinen Wunschträumen hingeben %74%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %27%; Mich vor dem Spiegel zurechtmachen %42%; Mich meinen Wunschträumen hingeben %74%; </t>
   </si>
   <si>
     <t>gadda.elena@web.te</t>
@@ -22622,7 +22622,7 @@
     <t>02341 47109</t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %10%; Jemanden beraten %46%; Jemandem behilflich sein %0%; Tagebuch schreiben %82%; Eine Dusche nehmen %46%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %10%; Jemanden beraten %46%; Jemandem behilflich sein %0%; Tagebuch schreiben %82%; Frische Luft schnappen %46%; </t>
   </si>
   <si>
     <t>elisabeth.flügemann@gmaiil.te</t>
@@ -23072,7 +23072,7 @@
     <t>04121 30906</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %44%; Für andere sorgen %1%; Am Ofen/Kamin sitzen, ins Feuer gucken %77%; Private Sachen erledigen, die schon lange liegengeblieben sind %97%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %44%; Für andere sorgen %1%; Am Ofen/Kamin sitzen, ins Feuer gucken %77%; Private Sachen erledigen, die schon lange liegengeblieben sind %97%; </t>
   </si>
   <si>
     <t>rolf.reismann@iunitimail.ork</t>
@@ -23351,7 +23351,7 @@
     <t>0202 / 643072</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine Dusche nehmen %5%; </t>
+    <t xml:space="preserve">Frische Luft schnappen %5%; </t>
   </si>
   <si>
     <t>franz-josef.bickmann@gmaiil.te</t>
@@ -23576,7 +23576,7 @@
     <t>05101 / 92119</t>
   </si>
   <si>
-    <t xml:space="preserve">Verabredungen treffen %34%; Computerspiele spielen %40%; Seine Haare waschen %0%; Etwas entwerfen oder zeichnen %96%; </t>
+    <t xml:space="preserve">Verabredungen treffen %34%; Computerspiele spielen %40%; Seine Fotos sortieren %0%; Etwas entwerfen oder zeichnen %96%; </t>
   </si>
   <si>
     <t>sven.maßmann@d-ohnline.kom</t>
@@ -23594,7 +23594,7 @@
     <t>07461 / 31024</t>
   </si>
   <si>
-    <t xml:space="preserve">Im Internet surfen %45%; Seine Haare waschen %40%; Etwas lernen und mich fortbilden %28%; </t>
+    <t xml:space="preserve">Im Internet surfen %45%; Seine Fotos sortieren %40%; Etwas lernen und mich fortbilden %28%; </t>
   </si>
   <si>
     <t>çolak.ayşe@gmaiil.te</t>
@@ -23792,7 +23792,7 @@
     <t>0203 / 915182</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich entspannen %10%; Eine Dusche nehmen %94%; </t>
+    <t xml:space="preserve">Sich entspannen %10%; Frische Luft schnappen %94%; </t>
   </si>
   <si>
     <t>carola.blümer@d-ohnline.te</t>
@@ -23807,7 +23807,7 @@
     <t>02173 1384</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %55%; Über meine Probleme reden %61%; Post lesen %21%; Die Bibel oder andere religiöse Schriften lesen %86%; </t>
+    <t xml:space="preserve">Für jemanden kochen %55%; Über meine Probleme reden %61%; Post lesen %21%; Die Bibel oder andere religiöse Schriften lesen %86%; </t>
   </si>
   <si>
     <t>20.02.1992</t>
@@ -24086,7 +24086,7 @@
     <t>0281 / 593438</t>
   </si>
   <si>
-    <t xml:space="preserve">Videos ansehen %4%; Ausgiebig baden %92%; Die Bibel oder andere religiöse Schriften lesen %83%; </t>
+    <t xml:space="preserve">Videos ansehen %4%; Ausgiebig Tee trinken %92%; Die Bibel oder andere religiöse Schriften lesen %83%; </t>
   </si>
   <si>
     <t>tomaszewski.janusz@gmaiil.te</t>
@@ -24116,7 +24116,7 @@
     <t>02227 21759</t>
   </si>
   <si>
-    <t xml:space="preserve">Fachliteratur oder Sachbuch lesen %59%; Eine Dusche nehmen %60%; </t>
+    <t xml:space="preserve">Fachliteratur oder Sachbuch lesen %59%; Frische Luft schnappen %60%; </t>
   </si>
   <si>
     <t>barbara.duday@gmaiil.te</t>
@@ -24209,7 +24209,7 @@
     <t>0611 / 431833</t>
   </si>
   <si>
-    <t xml:space="preserve">Ins Grüne fahren %69%; Sport treiben %43%; Mich nicht ausgenutzt fühlen %71%; Ausgiebig baden %83%; Etwas entwerfen oder zeichnen %63%; </t>
+    <t xml:space="preserve">Ins Grüne fahren %69%; Sport treiben %43%; Mich nicht ausgenutzt fühlen %71%; Ausgiebig Tee trinken %83%; Etwas entwerfen oder zeichnen %63%; </t>
   </si>
   <si>
     <t>annette.vennemann@ge-em-ix.te</t>
@@ -24599,7 +24599,7 @@
     <t>02943 / 66822</t>
   </si>
   <si>
-    <t xml:space="preserve">Massiert werden %4%; Jemandem eine Freude bereiten %27%; Mir selbst etwas kochen %8%; Mich meinen Wunschträumen hingeben %22%; </t>
+    <t xml:space="preserve">Von jemandem bekocht werden %4%; Jemandem eine Freude bereiten %27%; Mir selbst etwas kochen %8%; Mich meinen Wunschträumen hingeben %22%; </t>
   </si>
   <si>
     <t>constanze.hähn@d-ohnline.te</t>
@@ -24884,7 +24884,7 @@
     <t>(05431) 50396</t>
   </si>
   <si>
-    <t xml:space="preserve">Tanzen %59%; Um Hilfe und Ratschläge bitten %93%; Sich um neue Arbeit bewerben %100%; Eine Dusche nehmen %92%; </t>
+    <t xml:space="preserve">Tanzen %59%; Um Hilfe und Ratschläge bitten %93%; Sich um neue Arbeit bewerben %100%; Frische Luft schnappen %92%; </t>
   </si>
   <si>
     <t>hubert.patzek@web.te</t>
@@ -25004,7 +25004,7 @@
     <t>0461 / 914992</t>
   </si>
   <si>
-    <t xml:space="preserve">Kräuter/Pilze sammeln %73%; Ausgiebig frühstücken %76%; Eine Dusche nehmen %30%; </t>
+    <t xml:space="preserve">Kräuter/Pilze sammeln %73%; Ausgiebig frühstücken %76%; Frische Luft schnappen %30%; </t>
   </si>
   <si>
     <t>august.schulzehobeling@iunitimail.kom</t>
@@ -25118,7 +25118,7 @@
     <t>04331 / 96776</t>
   </si>
   <si>
-    <t xml:space="preserve">Gottesdienste besuchen %54%; Jemandem helfen %18%; Einfach alleine sein %50%; Eine Dusche nehmen %27%; </t>
+    <t xml:space="preserve">Gottesdienste besuchen %54%; Jemandem helfen %18%; Einfach alleine sein %50%; Frische Luft schnappen %27%; </t>
   </si>
   <si>
     <t>udo.schennen@d-ohnline.te</t>
@@ -25286,7 +25286,7 @@
     <t>06834 / 46436</t>
   </si>
   <si>
-    <t xml:space="preserve">Eine schwierige Aufgabe meistern %44%; Parfum benutzen %26%; Eine Dusche nehmen %36%; </t>
+    <t xml:space="preserve">Eine schwierige Aufgabe meistern %44%; Parfum benutzen %26%; Frische Luft schnappen %36%; </t>
   </si>
   <si>
     <t>allah.kamel@autluuk.kom</t>
@@ -25412,7 +25412,7 @@
     <t>(0241) 656860</t>
   </si>
   <si>
-    <t xml:space="preserve">Einen Vergnügungspark besuchen %100%; Über meine Arbeit reden %73%; Zeitschriften durchblättern/lesen %90%; Eine Dusche nehmen %9%; </t>
+    <t xml:space="preserve">Einen Vergnügungspark besuchen %100%; Über meine Arbeit reden %73%; Zeitschriften durchblättern/lesen %90%; Frische Luft schnappen %9%; </t>
   </si>
   <si>
     <t>heinz.gerstner@ge-em-ix.te</t>
@@ -25493,7 +25493,7 @@
     <t>(05275) 1405</t>
   </si>
   <si>
-    <t xml:space="preserve">E-Mails schreiben %79%; Seine Haare waschen %35%; Mit Bekannten telefonieren %73%; </t>
+    <t xml:space="preserve">E-Mails schreiben %79%; Seine Fotos sortieren %35%; Mit Bekannten telefonieren %73%; </t>
   </si>
   <si>
     <t>elisabeth.müller@web.te</t>
@@ -25619,7 +25619,7 @@
     <t>05232 / 14058</t>
   </si>
   <si>
-    <t xml:space="preserve">Jemanden massieren %22%; Computerspiele spielen %100%; Eine Anschaffung machen (Auto, Hausgegenstände, etc.) %41%; Ausschlafen %54%; </t>
+    <t xml:space="preserve">Für jemanden kochen %22%; Computerspiele spielen %100%; Eine Anschaffung machen (Auto, Hausgegenstände, etc.) %41%; Ausschlafen %54%; </t>
   </si>
   <si>
     <t>gutierrez.josefa@iunitimail.te</t>
@@ -26000,7 +26000,7 @@
     <t>(0491) 677114</t>
   </si>
   <si>
-    <t xml:space="preserve">Neue Bekanntschaften machen %45%; Seine Haare waschen %67%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %15%; </t>
+    <t xml:space="preserve">Neue Bekanntschaften machen %45%; Seine Fotos sortieren %67%; Lebensmittel einmachen, einfrieren, Vorräte anlegen %15%; </t>
   </si>
   <si>
     <t>yıldız.ceylan@d-ohnline.ork</t>
@@ -26147,7 +26147,7 @@
     <t>050 / 7348174</t>
   </si>
   <si>
-    <t xml:space="preserve">Einmal alleine wegfahren %89%; Schwierige Probleme klären %88%; Seine Haare waschen %72%; Auf mich zukommende Situationen in Gedanken bewältigen %17%; </t>
+    <t xml:space="preserve">Einmal alleine wegfahren %89%; Schwierige Probleme klären %88%; Seine Fotos sortieren %72%; Auf mich zukommende Situationen in Gedanken bewältigen %17%; </t>
   </si>
   <si>
     <t>martin.lemmer@gmaiil.ork</t>
@@ -26162,7 +26162,7 @@
     <t>(030) 2680002</t>
   </si>
   <si>
-    <t xml:space="preserve">Sich über Philosophie oder Religion unterhalten %62%; Kräuter/Pilze sammeln %88%; Eine Dusche nehmen %62%; </t>
+    <t xml:space="preserve">Sich über Philosophie oder Religion unterhalten %62%; Kräuter/Pilze sammeln %88%; Frische Luft schnappen %62%; </t>
   </si>
   <si>
     <t>walter.holtz@web.te</t>
@@ -26177,7 +26177,7 @@
     <t>0521 / 215141</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %67%; Für andere sorgen %7%; Fernsehen %82%; Für einen guten Zweck spenden %3%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %67%; Für andere sorgen %7%; Fernsehen %82%; Für einen guten Zweck spenden %3%; </t>
   </si>
   <si>
     <t>matthias.mönnighausen@iunitimail.ork</t>
@@ -26276,7 +26276,7 @@
     <t>(02041) 15103</t>
   </si>
   <si>
-    <t xml:space="preserve">Ein Musikinstrument spielen %99%; Ins Kino gehen %5%; Am Ofen/Kamin sitzen, ins Feuer gucken %59%; Eine Dusche nehmen %77%; </t>
+    <t xml:space="preserve">Ein Musikinstrument spielen %99%; Ins Kino gehen %5%; Am Ofen/Kamin sitzen, ins Feuer gucken %59%; Frische Luft schnappen %77%; </t>
   </si>
   <si>
     <t>tobias.bokel@d-ohnline.ork</t>
@@ -26291,7 +26291,7 @@
     <t>0211 / 248626</t>
   </si>
   <si>
-    <t xml:space="preserve">Computer-Netzwerk-Partys %95%; Ausgiebig baden %40%; Auf mich zukommende Situationen in Gedanken bewältigen %98%; </t>
+    <t xml:space="preserve">Computer-Netzwerk-Partys %95%; Ausgiebig Tee trinken %40%; Auf mich zukommende Situationen in Gedanken bewältigen %98%; </t>
   </si>
   <si>
     <t>ralf.burghoff@autluuk.kom</t>
@@ -26498,7 +26498,7 @@
     <t>0411 / 173366</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausflüge oder Urlaubsfahrten planen %37%; Reisen %56%; Ausgiebig baden %35%; Leger gekleidet sein %35%; </t>
+    <t xml:space="preserve">Ausflüge oder Urlaubsfahrten planen %37%; Reisen %56%; Ausgiebig Tee trinken %35%; Leger gekleidet sein %35%; </t>
   </si>
   <si>
     <t>karin.randow@iunitimail.ork</t>
@@ -26513,7 +26513,7 @@
     <t>02308 / 75168</t>
   </si>
   <si>
-    <t xml:space="preserve">Zum Zirkus oder Zoo gehen %65%; Massiert werden %55%; Meine Arbeit geschickt ausführen %59%; Seine finanziellen Angelegenheiten regeln %64%; Ein Nickerchen machen %76%; </t>
+    <t xml:space="preserve">Zum Zirkus oder Zoo gehen %65%; Von jemandem bekocht werden %55%; Meine Arbeit geschickt ausführen %59%; Seine finanziellen Angelegenheiten regeln %64%; Ein Nickerchen machen %76%; </t>
   </si>
   <si>
     <t>maria.engelmann@gmaiil.te</t>
@@ -26528,7 +26528,7 @@
     <t>(098) 6077391</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %79%; Streit aus dem Wege gehen %71%; An meine Freunde und Bekannten denken %37%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %79%; Streit aus dem Wege gehen %71%; An meine Freunde und Bekannten denken %37%; </t>
   </si>
   <si>
     <t>hildegard.wittkamp@d-ohnline.te</t>
@@ -26684,7 +26684,7 @@
     <t>0521 / 355256</t>
   </si>
   <si>
-    <t xml:space="preserve">Holz hacken %7%; Im Internet surfen %12%; Kreuzworträtsel lösen oder ein Puzzle legen %35%; Eine Dusche nehmen %26%; </t>
+    <t xml:space="preserve">Holz hacken %7%; Im Internet surfen %12%; Kreuzworträtsel lösen oder ein Puzzle legen %35%; Frische Luft schnappen %26%; </t>
   </si>
   <si>
     <t>ewald.mill@autluuk.te</t>
@@ -27080,7 +27080,7 @@
     <t>0211 / 288131</t>
   </si>
   <si>
-    <t xml:space="preserve">Zärtlich sein, schmusen, küssen %91%; Mit Partner oder Familie daheim sein %99%; Die Sterne oder den Mond beobachten %12%; Etwas planen oder organisieren %99%; </t>
+    <t xml:space="preserve">Einen gemütlichen Filmabend machen %91%; Mit Partner oder Familie daheim sein %99%; Die Sterne oder den Mond beobachten %12%; Etwas planen oder organisieren %99%; </t>
   </si>
   <si>
     <t>margarete.büll@web.te</t>
@@ -27113,7 +27113,7 @@
     <t>0511 / 504545</t>
   </si>
   <si>
-    <t xml:space="preserve">Computer-Netzwerk-Partys %68%; Mit Partner oder Familie daheim sein %71%; Stricken, Häkeln, Sticken oder Nähen %53%; Eine Dusche nehmen %32%; </t>
+    <t xml:space="preserve">Computer-Netzwerk-Partys %68%; Mit Partner oder Familie daheim sein %71%; Stricken, Häkeln, Sticken oder Nähen %53%; Frische Luft schnappen %32%; </t>
   </si>
   <si>
     <t>al-manfaluti.dschihan@gmaiil.te</t>
@@ -27791,7 +27791,7 @@
     <t>09772 / 36527</t>
   </si>
   <si>
-    <t xml:space="preserve">Parfum benutzen %5%; Eine Dusche nehmen %36%; </t>
+    <t xml:space="preserve">Parfum benutzen %5%; Frische Luft schnappen %36%; </t>
   </si>
   <si>
     <t>ebba.willems@web.te</t>
@@ -27896,7 +27896,7 @@
     <t>0201 / 171665</t>
   </si>
   <si>
-    <t xml:space="preserve">Mit seinem Partner zusammen sein %59%; Etwas fertig stellen %53%; Mir selbst etwas kochen %68%; Eine Dusche nehmen %40%; </t>
+    <t xml:space="preserve">Mit seinem Partner zusammen sein %59%; Etwas fertig stellen %53%; Mir selbst etwas kochen %68%; Frische Luft schnappen %40%; </t>
   </si>
   <si>
     <t>margot.beuse@web.te</t>
@@ -28100,7 +28100,7 @@
     <t xml:space="preserve">Landkarten studieren %1%; Netflix chillen %3%; An technischen Dingen arbeiten (Fahrzeuge, Hausgeräte usw.) %34%; </t>
   </si>
   <si>
-    <t xml:space="preserve">In die Sauna gehen %17%; Jemanden beraten %75%; Netflix chillen %99%; Mit Bekannten telefonieren %47%; </t>
+    <t xml:space="preserve">In die Bibliothek gehen %17%; Jemanden beraten %75%; Netflix chillen %99%; Mit Bekannten telefonieren %47%; </t>
   </si>
   <si>
     <t xml:space="preserve">Sich über Philosophie oder Religion unterhalten %33%; Mich nicht ausgenutzt fühlen %86%; Netflix chillen %96%; Romane, Erzählungen, Theaterstücke oder Gedichte schreiben %62%; </t>

</xml_diff>